<commit_message>
BBDD actualizada (12 emails nuevos) + primer contacto Apollo + rutina semanal
- Fusiona los 12 emails nuevos del Excel actualizado (quedan 55 municipios
  sin email) y limpia dos direcciones con punto final sobrante.
- Añade el primer contacto nominal verificado vía Apollo: Joan Campolier,
  Alcalde de Santa Susanna (demo del ciclo del agente).
- Documenta el modo principal de ejecución: Rutina de Claude semanal con
  los conectores de Apollo y HubSpot (pausada hasta arrancar la campaña);
  el workflow de GitHub Actions queda como alternativa con API key.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015oaFpSagWroLdzsbC55cuL
</commit_message>
<xml_diff>
--- a/data/ayuntamientos-costeros.xlsx
+++ b/data/ayuntamientos-costeros.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K224"/>
+  <dimension ref="A1:K225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1591,10 +1591,14 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>urbanisme@santpol.cat</t>
+        </is>
+      </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>No encontrado</t>
+          <t>Urbanismo</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1609,7 +1613,7 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
@@ -1677,10 +1681,14 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>massuettd@arenysdemar.cat</t>
+        </is>
+      </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>No encontrado</t>
+          <t>Urbanismo</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -1695,7 +1703,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
@@ -2148,10 +2156,14 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="2" t="inlineStr"/>
-      <c r="G39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>oac360@elprat.cat</t>
+        </is>
+      </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>No encontrado</t>
+          <t>Urbanismo</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
@@ -2166,7 +2178,7 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
@@ -2410,10 +2422,14 @@
       <c r="D45" s="2" t="inlineStr"/>
       <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="2" t="inlineStr"/>
-      <c r="G45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>urbanisme@vilanova.cat</t>
+        </is>
+      </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>No encontrado</t>
+          <t>Urbanismo</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -2428,7 +2444,7 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
@@ -5061,10 +5077,14 @@
       <c r="D104" s="2" t="inlineStr"/>
       <c r="E104" s="2" t="inlineStr"/>
       <c r="F104" s="2" t="inlineStr"/>
-      <c r="G104" s="2" t="inlineStr"/>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>participacio@altea.es</t>
+        </is>
+      </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>No encontrado</t>
+          <t>Urbanismo</t>
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr">
@@ -5079,7 +5099,7 @@
       </c>
       <c r="K104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
@@ -5462,7 +5482,11 @@
       <c r="D113" s="2" t="inlineStr"/>
       <c r="E113" s="2" t="inlineStr"/>
       <c r="F113" s="2" t="inlineStr"/>
-      <c r="G113" s="2" t="inlineStr"/>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>urbanismo@torrevieja.eu</t>
+        </is>
+      </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
           <t>No encontrado</t>
@@ -5480,7 +5504,7 @@
       </c>
       <c r="K113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
@@ -5634,10 +5658,14 @@
       <c r="D117" s="2" t="inlineStr"/>
       <c r="E117" s="2" t="inlineStr"/>
       <c r="F117" s="2" t="inlineStr"/>
-      <c r="G117" s="2" t="inlineStr"/>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>calvia@calvia.com</t>
+        </is>
+      </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>No encontrado</t>
+          <t>Urbanismo</t>
         </is>
       </c>
       <c r="I117" s="2" t="inlineStr">
@@ -5652,7 +5680,7 @@
       </c>
       <c r="K117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
@@ -5900,10 +5928,14 @@
       <c r="D123" s="2" t="inlineStr"/>
       <c r="E123" s="2" t="inlineStr"/>
       <c r="F123" s="2" t="inlineStr"/>
-      <c r="G123" s="2" t="inlineStr"/>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>mediambient@a-soller.es</t>
+        </is>
+      </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t>No encontrado</t>
+          <t>Medioambiente</t>
         </is>
       </c>
       <c r="I123" s="2" t="inlineStr">
@@ -5918,7 +5950,7 @@
       </c>
       <c r="K123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
@@ -5986,10 +6018,14 @@
       <c r="D125" s="2" t="inlineStr"/>
       <c r="E125" s="2" t="inlineStr"/>
       <c r="F125" s="2" t="inlineStr"/>
-      <c r="G125" s="2" t="inlineStr"/>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>mediambient@ajpollenca.net</t>
+        </is>
+      </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>No encontrado</t>
+          <t>Medioambiente</t>
         </is>
       </c>
       <c r="I125" s="2" t="inlineStr">
@@ -6004,7 +6040,7 @@
       </c>
       <c r="K125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
@@ -6027,10 +6063,14 @@
       <c r="D126" s="2" t="inlineStr"/>
       <c r="E126" s="2" t="inlineStr"/>
       <c r="F126" s="2" t="inlineStr"/>
-      <c r="G126" s="2" t="inlineStr"/>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>emsa@alcudia.net</t>
+        </is>
+      </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>No encontrado</t>
+          <t>Medioambiente</t>
         </is>
       </c>
       <c r="I126" s="2" t="inlineStr">
@@ -6045,7 +6085,7 @@
       </c>
       <c r="K126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
@@ -6068,10 +6108,14 @@
       <c r="D127" s="2" t="inlineStr"/>
       <c r="E127" s="2" t="inlineStr"/>
       <c r="F127" s="2" t="inlineStr"/>
-      <c r="G127" s="2" t="inlineStr"/>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>mediambient@vilademuro.net</t>
+        </is>
+      </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>No encontrado</t>
+          <t>Medioambiente</t>
         </is>
       </c>
       <c r="I127" s="2" t="inlineStr">
@@ -6086,7 +6130,7 @@
       </c>
       <c r="K127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
@@ -6322,10 +6366,14 @@
       <c r="D133" s="2" t="inlineStr"/>
       <c r="E133" s="2" t="inlineStr"/>
       <c r="F133" s="2" t="inlineStr"/>
-      <c r="G133" s="2" t="inlineStr"/>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>consultesurbanisme@manacor.org</t>
+        </is>
+      </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
-          <t>No encontrado</t>
+          <t>Urbanismo</t>
         </is>
       </c>
       <c r="I133" s="2" t="inlineStr">
@@ -6340,7 +6388,7 @@
       </c>
       <c r="K133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
@@ -10260,6 +10308,63 @@
       <c r="K224" s="2" t="inlineStr">
         <is>
           <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>Santa Susanna</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="E225" s="2" t="inlineStr">
+        <is>
+          <t>Campolier</t>
+        </is>
+      </c>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="G225" s="2" t="inlineStr">
+        <is>
+          <t>ajuntament@stasusanna.org</t>
+        </is>
+      </c>
+      <c r="H225" s="2" t="inlineStr">
+        <is>
+          <t>General (nominal · verificado Apollo)</t>
+        </is>
+      </c>
+      <c r="I225" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/joan-campolier-bb9a5027</t>
+        </is>
+      </c>
+      <c r="J225" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K225" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
@@ -10310,7 +10415,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>156</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5">
@@ -10320,7 +10425,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>67</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6">
@@ -10330,7 +10435,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>156</v>
+        <v>169</v>
       </c>
     </row>
     <row r="7">
@@ -10340,7 +10445,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -10355,7 +10460,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Prueba real del ciclo semanal: Lucia Cuesta (Ajuntament de Barcelona)
Recorrido de la rotación Caldes d'Estrac → Vilassar de Mar → Montgat →
Sant Adrià → Barcelona; solo Barcelona tenía contacto con email disponible.
Añadida a la lista OUTBOUND - MOBILIARIO URBANO de Apollo, al CSV/Excel y a
HubSpot. La organización de Barcelona figura en Apollo como «Barcelona City
Council», así que se añade esa variante a la búsqueda del agente.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015oaFpSagWroLdzsbC55cuL
</commit_message>
<xml_diff>
--- a/data/ayuntamientos-costeros.xlsx
+++ b/data/ayuntamientos-costeros.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K225"/>
+  <dimension ref="A1:K226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -10363,6 +10363,63 @@
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>Lucia</t>
+        </is>
+      </c>
+      <c r="E226" s="2" t="inlineStr">
+        <is>
+          <t>Cuesta Fernandez</t>
+        </is>
+      </c>
+      <c r="F226" s="2" t="inlineStr">
+        <is>
+          <t>Técnica de Medio Ambiente y Costas</t>
+        </is>
+      </c>
+      <c r="G226" s="2" t="inlineStr">
+        <is>
+          <t>lucia.fernandez@barcelona.cat</t>
+        </is>
+      </c>
+      <c r="H226" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I226" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/lucia-cuesta-fernández-388a2366</t>
+        </is>
+      </c>
+      <c r="J226" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K226" s="2" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
@@ -10415,7 +10472,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5">
@@ -10425,7 +10482,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6">
@@ -10435,7 +10492,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7">
@@ -10445,7 +10502,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Segunda verificación del agente: Héctor Pons, Alcalde de Maó
Lote Viladecans→Felanitx sin emails enriquecibles; la búsqueda agrupada por
dominios del lote encontró al alcalde de Maó (municipio sin email en la
BBDD). Añadido a la lista OUTBOUND, al CSV/Excel y a HubSpot.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015oaFpSagWroLdzsbC55cuL
</commit_message>
<xml_diff>
--- a/data/ayuntamientos-costeros.xlsx
+++ b/data/ayuntamientos-costeros.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K226"/>
+  <dimension ref="A1:K227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -10420,6 +10420,63 @@
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>Maó</t>
+        </is>
+      </c>
+      <c r="B227" s="2" t="inlineStr">
+        <is>
+          <t>Illes Balears</t>
+        </is>
+      </c>
+      <c r="C227" s="2" t="inlineStr">
+        <is>
+          <t>Islas Baleares</t>
+        </is>
+      </c>
+      <c r="D227" s="2" t="inlineStr">
+        <is>
+          <t>Hector</t>
+        </is>
+      </c>
+      <c r="E227" s="2" t="inlineStr">
+        <is>
+          <t>Pons Riudavets</t>
+        </is>
+      </c>
+      <c r="F227" s="2" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="G227" s="2" t="inlineStr">
+        <is>
+          <t>hpons@ajmao.org</t>
+        </is>
+      </c>
+      <c r="H227" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I227" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/hectorpons</t>
+        </is>
+      </c>
+      <c r="J227" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K227" s="2" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
@@ -10472,7 +10529,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5">
@@ -10482,7 +10539,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6">
@@ -10492,7 +10549,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7">
@@ -10502,7 +10559,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Ejecución semanal 2026-S37: Juan Martel (Ayuntamiento de Telde)
Lote de 25 municipios de Baleares y Canarias sin email. Búsqueda agrupada
por dominios: 1 contacto válido (Telde, verificado por dominio) y 1
descartado por la regla de calidad (técnica del Cabildo de Tenerife, no es
un ayuntamiento de la BBDD). Añadido a la lista OUTBOUND, al CSV/Excel y a
HubSpot. Créditos gastados: 1.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015oaFpSagWroLdzsbC55cuL
</commit_message>
<xml_diff>
--- a/data/ayuntamientos-costeros.xlsx
+++ b/data/ayuntamientos-costeros.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K227"/>
+  <dimension ref="A1:K228"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -10479,6 +10479,63 @@
       <c r="K227" s="2" t="inlineStr">
         <is>
           <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>Telde</t>
+        </is>
+      </c>
+      <c r="B228" s="2" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="inlineStr">
+        <is>
+          <t>Canarias</t>
+        </is>
+      </c>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>Juan</t>
+        </is>
+      </c>
+      <c r="E228" s="2" t="inlineStr">
+        <is>
+          <t>Martel</t>
+        </is>
+      </c>
+      <c r="F228" s="2" t="inlineStr">
+        <is>
+          <t>Segundo Teniente Alcalde y Concejal de Vías y Obras</t>
+        </is>
+      </c>
+      <c r="G228" s="2" t="inlineStr">
+        <is>
+          <t>juanmartel@telde.es</t>
+        </is>
+      </c>
+      <c r="H228" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I228" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/juan-martel-santana-99501099</t>
+        </is>
+      </c>
+      <c r="J228" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K228" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
         </is>
       </c>
     </row>
@@ -10529,7 +10586,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5">
@@ -10539,7 +10596,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6">
@@ -10549,7 +10606,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="7">
@@ -10559,7 +10616,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -10574,7 +10631,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-07</t>
         </is>
       </c>
     </row>

</xml_diff>